<commit_message>
updated dialogue for found items
</commit_message>
<xml_diff>
--- a/dialogue.xlsx
+++ b/dialogue.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\noorb\Documents\GitHub\Nut-Digger\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAF70E80-044C-49A7-B92E-3CBDD52F15F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FD5FBB6-696F-4B53-80E7-E9617C53B5A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{5407D05E-54CC-46DD-837F-C8BB1BCABA22}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="75">
   <si>
     <t>name</t>
   </si>
@@ -171,9 +171,6 @@
     <t>I want to bet, money tips?</t>
   </si>
   <si>
-    <t>"You know I heard about a golden ring in the dark forest, I'll give you 1k nuts for it.","You get the ring yet brokie?"</t>
-  </si>
-  <si>
     <t>"Wow I didn't think you'd actually go get it" -&gt; special trigger</t>
   </si>
   <si>
@@ -222,17 +219,29 @@
     <t>Billies house</t>
   </si>
   <si>
-    <t>picture frame</t>
-  </si>
-  <si>
     <t>"A family picture in front of a large lake"</t>
   </si>
   <si>
     <t>hidden newspaper snippet</t>
   </si>
   <si>
+    <t>"note to passerby: if Francis is lost again, tell him to look for the big arrow."</t>
+  </si>
+  <si>
+    <t>"You know I heard about a golden ring in the dark forest, I'll give you 1k nuts for it, or you can use it to marry some rich idiot hahaha","You get the ring yet brokie?"</t>
+  </si>
+  <si>
+    <t>Large picture frame</t>
+  </si>
+  <si>
+    <t>hiking gear on the wall</t>
+  </si>
+  <si>
+    <t>"Hiking gear, it looks expensive"</t>
+  </si>
+  <si>
     <r>
-      <t>"</t>
+      <t xml:space="preserve">"1980: </t>
     </r>
     <r>
       <rPr>
@@ -257,13 +266,28 @@
     </r>
   </si>
   <si>
-    <t>picture lying on table</t>
-  </si>
-  <si>
-    <t>"An old picture, Billie is wearing a suit and speaking on the phone"</t>
-  </si>
-  <si>
-    <t>"note to passerby: if Francis is lost again, tell him to look for the big arrow."</t>
+    <t>teaset next to couch</t>
+  </si>
+  <si>
+    <t>"A fine china teaset, the cups have golden rims"</t>
+  </si>
+  <si>
+    <t>pipe</t>
+  </si>
+  <si>
+    <t>picture on the wall</t>
+  </si>
+  <si>
+    <t>"An old picture, a serious Billie is wearing a suit and speaking on the phone"</t>
+  </si>
+  <si>
+    <t>"A strange pipe"</t>
+  </si>
+  <si>
+    <t>meds on the table</t>
+  </si>
+  <si>
+    <t>"Some Voltaren and Ibuprofen"</t>
   </si>
 </sst>
 </file>
@@ -759,7 +783,7 @@
         <v>26</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>43</v>
+        <v>62</v>
       </c>
       <c r="F5" s="1"/>
       <c r="G5" s="1"/>
@@ -808,16 +832,16 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="C9" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="D9" s="1" t="s">
         <v>47</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="72.5" x14ac:dyDescent="0.35">
@@ -834,7 +858,7 @@
         <v>38</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
@@ -875,7 +899,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F3D1FD7-5624-443C-86A7-B25899C382C7}">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18.453125" customWidth="1"/>
@@ -885,68 +909,112 @@
   <sheetData>
     <row r="1" spans="1:3" ht="16" x14ac:dyDescent="0.4">
       <c r="A1" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>49</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C2" t="s">
         <v>53</v>
-      </c>
-      <c r="C2" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>56</v>
-      </c>
       <c r="C3" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B4" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B5" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B6" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="29" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>57</v>
+      </c>
+      <c r="B7" t="s">
+        <v>67</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>58</v>
+      </c>
+      <c r="B8" t="s">
+        <v>70</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>58</v>
+      </c>
+      <c r="B9" t="s">
+        <v>69</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>58</v>
+      </c>
+      <c r="B10" t="s">
+        <v>73</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>